<commit_message>
Signed-off-by: Student Jack O Mahoney (TL_KCOMP_B_Y3) <t00261288@mymtu.ie>
</commit_message>
<xml_diff>
--- a/Assignment 1 JOM.xlsx
+++ b/Assignment 1 JOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentJackOMahoney(\Desktop\CG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD28B7EB-240A-4ECB-B981-5CF580652C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB24F785-F9B9-4270-A9F6-6A07916B09C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -559,44 +559,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -928,6 +928,270 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>848516</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>3362739</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{630DABD5-8D72-6170-F02B-992845EA20FF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8191500" y="22296783"/>
+          <a:ext cx="2687255" cy="3362739"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>33131</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>82</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B9CBF439-6F12-D50F-AF52-7673496AAA46}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8191500" y="13558630"/>
+          <a:ext cx="1871870" cy="1184495"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2465294</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>1425363</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FD91FD01-ADCF-06E4-BB3B-DE12118428DE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1815353" y="27678530"/>
+          <a:ext cx="2465294" cy="1425362"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1245692</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>4493559</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D1D2371F-C81A-7B18-5D2B-325006D01280}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1815353" y="29426647"/>
+          <a:ext cx="3755810" cy="4493559"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1102730</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>2028265</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{798CF75B-994B-1AAB-B6E9-5C5DA898E32B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1815353" y="34939941"/>
+          <a:ext cx="3612848" cy="2028265"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>22411</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>145676</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2644587</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>1413096</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D069118-DC5A-F019-D064-799E3D13F283}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11777382" y="27667323"/>
+          <a:ext cx="2622176" cy="1424302"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1231,24 +1495,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
@@ -1630,10 +1894,10 @@
     </row>
     <row r="2" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C2" s="4"/>
-      <c r="D2" s="42" t="s">
+      <c r="D2" s="46" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="43"/>
+      <c r="E2" s="47"/>
       <c r="F2" s="7"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -1644,8 +1908,8 @@
     </row>
     <row r="3" spans="3:13" ht="408.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C3" s="4"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="41"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="40"/>
       <c r="F3" s="5"/>
       <c r="G3" s="10"/>
       <c r="H3" s="6"/>
@@ -1665,10 +1929,10 @@
     </row>
     <row r="5" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="4"/>
-      <c r="D5" s="42" t="s">
+      <c r="D5" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="43"/>
+      <c r="E5" s="47"/>
       <c r="F5" s="7"/>
       <c r="H5" s="14"/>
       <c r="I5" s="11"/>
@@ -1677,8 +1941,8 @@
     </row>
     <row r="6" spans="3:13" ht="138.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C6" s="4"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="41"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="40"/>
       <c r="F6" s="15"/>
       <c r="G6" s="11"/>
       <c r="H6" s="14"/>
@@ -1698,10 +1962,10 @@
     </row>
     <row r="8" spans="3:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="4"/>
-      <c r="D8" s="42" t="s">
+      <c r="D8" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="43"/>
+      <c r="E8" s="47"/>
       <c r="F8" s="16"/>
       <c r="G8" s="11"/>
       <c r="H8" s="14"/>
@@ -1711,8 +1975,8 @@
     </row>
     <row r="9" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C9" s="4"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="41"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="40"/>
       <c r="F9" s="16"/>
       <c r="G9" s="11"/>
       <c r="H9" s="14"/>
@@ -1732,10 +1996,10 @@
     </row>
     <row r="11" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C11" s="4"/>
-      <c r="D11" s="42" t="s">
+      <c r="D11" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="E11" s="43"/>
+      <c r="E11" s="47"/>
       <c r="F11" s="17"/>
       <c r="G11" s="18"/>
       <c r="H11" s="44" t="s">
@@ -1748,12 +2012,12 @@
     </row>
     <row r="12" spans="3:13" ht="93" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C12" s="4"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="41"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="40"/>
       <c r="F12" s="15"/>
       <c r="G12" s="15"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="41"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="40"/>
       <c r="J12" s="15"/>
       <c r="K12" s="11"/>
       <c r="L12" s="14"/>
@@ -1773,10 +2037,10 @@
     </row>
     <row r="14" spans="3:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C14" s="4"/>
-      <c r="D14" s="42" t="s">
+      <c r="D14" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="E14" s="43"/>
+      <c r="E14" s="47"/>
       <c r="F14" s="16"/>
       <c r="G14" s="11"/>
       <c r="H14" s="14"/>
@@ -1788,8 +2052,8 @@
     </row>
     <row r="15" spans="3:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C15" s="4"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="41"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="40"/>
       <c r="F15" s="16"/>
       <c r="G15" s="11"/>
       <c r="H15" s="14"/>
@@ -1813,10 +2077,10 @@
     </row>
     <row r="17" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C17" s="4"/>
-      <c r="D17" s="42" t="s">
+      <c r="D17" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="E17" s="43"/>
+      <c r="E17" s="47"/>
       <c r="F17" s="17"/>
       <c r="G17" s="11"/>
       <c r="H17" s="14"/>
@@ -1828,8 +2092,8 @@
     </row>
     <row r="18" spans="1:13" ht="107.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C18" s="4"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="41"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="40"/>
       <c r="F18" s="19"/>
       <c r="H18" s="14"/>
       <c r="I18" s="11"/>
@@ -1850,14 +2114,14 @@
     </row>
     <row r="20" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C20" s="4"/>
-      <c r="D20" s="42" t="s">
+      <c r="D20" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="43"/>
-      <c r="F20" s="46" t="s">
+      <c r="E20" s="47"/>
+      <c r="F20" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="G20" s="47"/>
+      <c r="G20" s="43"/>
       <c r="H20" s="44" t="s">
         <v>1</v>
       </c>
@@ -1869,12 +2133,12 @@
     </row>
     <row r="21" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C21" s="4"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="41"/>
-      <c r="F21" s="46"/>
-      <c r="G21" s="47"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="41"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="41"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="40"/>
       <c r="J21" s="16"/>
       <c r="K21" s="11"/>
       <c r="L21" s="14"/>
@@ -1892,10 +2156,10 @@
     </row>
     <row r="23" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C23" s="4"/>
-      <c r="D23" s="42" t="s">
+      <c r="D23" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="43"/>
+      <c r="E23" s="47"/>
       <c r="F23" s="8"/>
       <c r="G23" s="21"/>
       <c r="H23" s="21"/>
@@ -1909,16 +2173,16 @@
     </row>
     <row r="24" spans="1:13" ht="113.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C24" s="4"/>
-      <c r="D24" s="40"/>
-      <c r="E24" s="41"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="40"/>
       <c r="F24" s="5"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
       <c r="I24" s="10"/>
       <c r="J24" s="6"/>
       <c r="K24" s="22"/>
-      <c r="L24" s="40"/>
-      <c r="M24" s="41"/>
+      <c r="L24" s="38"/>
+      <c r="M24" s="40"/>
     </row>
     <row r="25" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D25" s="12"/>
@@ -1945,8 +2209,8 @@
       <c r="A27" s="4"/>
       <c r="B27" s="5"/>
       <c r="C27" s="6"/>
-      <c r="D27" s="40"/>
-      <c r="E27" s="41"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="40"/>
       <c r="F27" s="11"/>
       <c r="J27" s="14"/>
       <c r="K27" s="11"/>
@@ -1969,10 +2233,10 @@
       </c>
       <c r="B29" s="45"/>
       <c r="C29" s="24"/>
-      <c r="D29" s="42" t="s">
+      <c r="D29" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="43"/>
+      <c r="E29" s="47"/>
       <c r="F29" s="8"/>
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
@@ -1983,11 +2247,11 @@
       <c r="M29" s="11"/>
     </row>
     <row r="30" spans="1:13" ht="322.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="40"/>
-      <c r="B30" s="41"/>
+      <c r="A30" s="38"/>
+      <c r="B30" s="40"/>
       <c r="C30" s="24"/>
-      <c r="D30" s="40"/>
-      <c r="E30" s="41"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="40"/>
       <c r="F30" s="19"/>
       <c r="G30" s="20"/>
       <c r="H30" s="20"/>
@@ -2005,44 +2269,44 @@
       <c r="M31" s="7"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A32" s="42" t="s">
+      <c r="A32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="43"/>
+      <c r="B32" s="47"/>
       <c r="C32" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="42" t="s">
+      <c r="D32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="E32" s="43"/>
-      <c r="F32" s="46" t="s">
+      <c r="E32" s="47"/>
+      <c r="F32" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="G32" s="49"/>
-      <c r="H32" s="49"/>
-      <c r="I32" s="49"/>
-      <c r="J32" s="49"/>
-      <c r="K32" s="47"/>
-      <c r="L32" s="42" t="s">
+      <c r="G32" s="42"/>
+      <c r="H32" s="42"/>
+      <c r="I32" s="42"/>
+      <c r="J32" s="42"/>
+      <c r="K32" s="43"/>
+      <c r="L32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="M32" s="43"/>
+      <c r="M32" s="47"/>
     </row>
     <row r="33" spans="1:13" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="50"/>
-      <c r="B33" s="48"/>
+      <c r="A33" s="48"/>
+      <c r="B33" s="39"/>
       <c r="C33" s="16"/>
-      <c r="D33" s="40"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="46"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="47"/>
-      <c r="L33" s="40"/>
-      <c r="M33" s="48"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="41"/>
+      <c r="G33" s="42"/>
+      <c r="H33" s="42"/>
+      <c r="I33" s="42"/>
+      <c r="J33" s="42"/>
+      <c r="K33" s="43"/>
+      <c r="L33" s="38"/>
+      <c r="M33" s="39"/>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="20"/>
@@ -2062,38 +2326,25 @@
     </row>
     <row r="36" spans="1:13" ht="213.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C36" s="4"/>
-      <c r="D36" s="40"/>
-      <c r="E36" s="41"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="40"/>
       <c r="F36" s="11"/>
     </row>
     <row r="38" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E38" s="25"/>
       <c r="F38" s="25"/>
-      <c r="H38" s="40"/>
-      <c r="I38" s="48"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="39"/>
     </row>
     <row r="91" ht="0.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F32:K32"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:K33"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="L32:M32"/>
-    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D8:E8"/>
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H11:I11"/>
@@ -2110,12 +2361,25 @@
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="L33:M33"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="F32:K32"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:K33"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="D32:E32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>